<commit_message>
Add 'verhuizingTijdGemeldNaVerzoek' attribute to casus Excel
</commit_message>
<xml_diff>
--- a/casus hackaton.xlsx
+++ b/casus hackaton.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pascal/projects/quintor/svb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\svb-hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9339D68B-8019-8F4C-BF6F-A714898C7750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5694AAD-2D75-46F7-B0AD-A82C35FF726E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="36000" windowHeight="22580" xr2:uid="{80954343-1134-47C3-8762-FA936ED9CB61}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80954343-1134-47C3-8762-FA936ED9CB61}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="87">
   <si>
     <t>de beoordelingsdatum</t>
   </si>
@@ -297,6 +297,9 @@
   </si>
   <si>
     <t>beleidsvoorbeeldEmotioneleOntwrichting</t>
+  </si>
+  <si>
+    <t>verhuizingTijdigGemeldNaVerzoek</t>
   </si>
 </sst>
 </file>
@@ -731,17 +734,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B301B29-CF91-4A5C-89D9-2D598FBE3789}">
   <dimension ref="A1:F150"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="81.33203125" customWidth="1"/>
-    <col min="4" max="4" width="46.83203125" customWidth="1"/>
+    <col min="4" max="4" width="46.77734375" customWidth="1"/>
     <col min="5" max="5" width="36.33203125" customWidth="1"/>
-    <col min="6" max="6" width="49.1640625" customWidth="1"/>
+    <col min="6" max="6" width="49.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="6"/>
       <c r="B1" s="6" t="s">
         <v>57</v>
@@ -759,12 +762,12 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C2" s="8"/>
       <c r="D2" s="3"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>40</v>
       </c>
@@ -773,7 +776,7 @@
       <c r="D3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C4" s="8" t="s">
         <v>0</v>
       </c>
@@ -787,7 +790,7 @@
         <v>46287</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>56</v>
       </c>
@@ -804,7 +807,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
@@ -812,7 +815,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
@@ -820,7 +823,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C8" s="8" t="s">
         <v>8</v>
       </c>
@@ -828,7 +831,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>59</v>
       </c>
@@ -845,7 +848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>58</v>
       </c>
@@ -862,7 +865,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>85</v>
       </c>
@@ -879,7 +882,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>60</v>
       </c>
@@ -896,7 +899,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C13" s="8" t="s">
         <v>11</v>
       </c>
@@ -904,7 +907,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>61</v>
       </c>
@@ -921,7 +924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C15" s="8" t="s">
         <v>12</v>
       </c>
@@ -929,7 +932,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>62</v>
       </c>
@@ -946,7 +949,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C17" s="8" t="s">
         <v>17</v>
       </c>
@@ -954,7 +957,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C18" s="8" t="s">
         <v>18</v>
       </c>
@@ -962,7 +965,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>63</v>
       </c>
@@ -979,7 +982,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>64</v>
       </c>
@@ -994,7 +997,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>65</v>
       </c>
@@ -1011,7 +1014,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>66</v>
       </c>
@@ -1028,7 +1031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:6" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:6" ht="31.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>67</v>
       </c>
@@ -1045,7 +1048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="31.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:6" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C24" s="8" t="s">
         <v>23</v>
       </c>
@@ -1053,7 +1056,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C25" s="8" t="s">
         <v>24</v>
       </c>
@@ -1061,7 +1064,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>68</v>
       </c>
@@ -1076,7 +1079,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>69</v>
       </c>
@@ -1093,7 +1096,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>70</v>
       </c>
@@ -1110,7 +1113,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>71</v>
       </c>
@@ -1127,7 +1130,10 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>86</v>
+      </c>
       <c r="C30" s="8" t="s">
         <v>31</v>
       </c>
@@ -1135,7 +1141,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>72</v>
       </c>
@@ -1152,7 +1158,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="2:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>73</v>
       </c>
@@ -1169,7 +1175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>74</v>
       </c>
@@ -1184,7 +1190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>75</v>
       </c>
@@ -1201,7 +1207,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>76</v>
       </c>
@@ -1218,7 +1224,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>77</v>
       </c>
@@ -1235,7 +1241,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>78</v>
       </c>
@@ -1252,7 +1258,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C38" s="8" t="s">
         <v>43</v>
       </c>
@@ -1260,7 +1266,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
       <c r="B39" s="12" t="s">
         <v>79</v>
@@ -1278,7 +1284,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B40" s="12" t="s">
         <v>80</v>
       </c>
@@ -1295,7 +1301,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B41" s="12" t="s">
         <v>81</v>
       </c>
@@ -1312,7 +1318,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B42" s="12" t="s">
         <v>82</v>
       </c>
@@ -1329,18 +1335,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C44" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C45" s="8" t="s">
         <v>51</v>
       </c>
@@ -1351,11 +1357,11 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>38</v>
       </c>
@@ -1364,7 +1370,7 @@
       <c r="D47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>39</v>
       </c>
@@ -1384,7 +1390,7 @@
         <v>42454</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>39</v>
       </c>
@@ -1397,7 +1403,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>55</v>
       </c>
@@ -1417,7 +1423,7 @@
         <v>43191</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>55</v>
       </c>
@@ -1430,403 +1436,403 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="10"/>
       <c r="D52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="8"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
     </row>

</xml_diff>

<commit_message>
Create rule for D112
</commit_message>
<xml_diff>
--- a/casus hackaton.xlsx
+++ b/casus hackaton.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\svb-hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5694AAD-2D75-46F7-B0AD-A82C35FF726E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B199DA79-7990-4A8A-B73F-7B05FC0A3488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80954343-1134-47C3-8762-FA936ED9CB61}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="88">
   <si>
     <t>de beoordelingsdatum</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t>verhuizingTijdigGemeldNaVerzoek</t>
+  </si>
+  <si>
+    <t>uitkeringKanHerleven</t>
   </si>
 </sst>
 </file>
@@ -1259,6 +1262,9 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B38" t="s">
+        <v>87</v>
+      </c>
       <c r="C38" s="8" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Create rule for D113111
</commit_message>
<xml_diff>
--- a/casus hackaton.xlsx
+++ b/casus hackaton.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\svb-hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B199DA79-7990-4A8A-B73F-7B05FC0A3488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAF9C9D-3CBE-4C51-A242-D85D654BE9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80954343-1134-47C3-8762-FA936ED9CB61}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="90">
   <si>
     <t>de beoordelingsdatum</t>
   </si>
@@ -303,6 +303,12 @@
   </si>
   <si>
     <t>uitkeringKanHerleven</t>
+  </si>
+  <si>
+    <t>voorzieneOmstandigheid</t>
+  </si>
+  <si>
+    <t>gewensteOmstandigheid</t>
   </si>
 </sst>
 </file>
@@ -811,6 +817,9 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
       <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
@@ -819,6 +828,9 @@
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>88</v>
+      </c>
       <c r="C7" s="8" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Create rule for D11311
</commit_message>
<xml_diff>
--- a/casus hackaton.xlsx
+++ b/casus hackaton.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Code\svb-hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAF9C9D-3CBE-4C51-A242-D85D654BE9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA1BCAE-82EE-4380-BD12-127B5245AD1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80954343-1134-47C3-8762-FA936ED9CB61}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="91">
   <si>
     <t>de beoordelingsdatum</t>
   </si>
@@ -309,6 +309,9 @@
   </si>
   <si>
     <t>gewensteOmstandigheid</t>
+  </si>
+  <si>
+    <t>nakomenFeitelijkOnmogelijk</t>
   </si>
 </sst>
 </file>
@@ -839,6 +842,9 @@
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
       <c r="C8" s="8" t="s">
         <v>8</v>
       </c>

</xml_diff>